<commit_message>
finished excel creation, need to modify docx and template
</commit_message>
<xml_diff>
--- a/.claude/skills/per-option-value/template/ESO multi-batch.xlsx
+++ b/.claude/skills/per-option-value/template/ESO multi-batch.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\tommy\Documents\Github\simple-agent\.claude\skills\per-option-value\template\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BF4590BF-9339-439A-B170-6D8ECE9A037F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0A231008-6970-46CD-AAC9-F6FAEB63A865}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-825" yWindow="1230" windowWidth="13920" windowHeight="11385" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="420" yWindow="2100" windowWidth="13920" windowHeight="11385" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="ESO" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="91" uniqueCount="71">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="75" uniqueCount="70">
   <si>
     <t>In HKD unless otherwise stated in this worksheet</t>
     <phoneticPr fontId="0" type="noConversion"/>
@@ -244,9 +244,6 @@
   </si>
   <si>
     <t>{{No. of Share Options2}}</t>
-  </si>
-  <si>
-    <t>…</t>
   </si>
   <si>
     <t>{{PerOptionValue1}}</t>
@@ -444,7 +441,7 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="56">
+  <cellXfs count="55">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
@@ -539,9 +536,6 @@
     </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="2" fontId="12" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
@@ -574,13 +568,13 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>10</xdr:col>
+      <xdr:col>9</xdr:col>
       <xdr:colOff>840442</xdr:colOff>
       <xdr:row>79</xdr:row>
       <xdr:rowOff>22412</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>16</xdr:col>
+      <xdr:col>15</xdr:col>
       <xdr:colOff>398307</xdr:colOff>
       <xdr:row>89</xdr:row>
       <xdr:rowOff>22412</xdr:rowOff>
@@ -618,13 +612,13 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>11</xdr:col>
+      <xdr:col>10</xdr:col>
       <xdr:colOff>11206</xdr:colOff>
       <xdr:row>31</xdr:row>
       <xdr:rowOff>11206</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>14</xdr:col>
+      <xdr:col>13</xdr:col>
       <xdr:colOff>532455</xdr:colOff>
       <xdr:row>37</xdr:row>
       <xdr:rowOff>20587</xdr:rowOff>
@@ -662,13 +656,13 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>11</xdr:col>
+      <xdr:col>10</xdr:col>
       <xdr:colOff>11205</xdr:colOff>
       <xdr:row>69</xdr:row>
       <xdr:rowOff>11207</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>14</xdr:col>
+      <xdr:col>13</xdr:col>
       <xdr:colOff>686984</xdr:colOff>
       <xdr:row>77</xdr:row>
       <xdr:rowOff>33619</xdr:rowOff>
@@ -706,13 +700,13 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>11</xdr:col>
+      <xdr:col>10</xdr:col>
       <xdr:colOff>44823</xdr:colOff>
       <xdr:row>116</xdr:row>
       <xdr:rowOff>33617</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>20</xdr:col>
+      <xdr:col>19</xdr:col>
       <xdr:colOff>37143</xdr:colOff>
       <xdr:row>150</xdr:row>
       <xdr:rowOff>61379</xdr:rowOff>
@@ -750,13 +744,13 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>11</xdr:col>
+      <xdr:col>10</xdr:col>
       <xdr:colOff>33616</xdr:colOff>
       <xdr:row>91</xdr:row>
       <xdr:rowOff>22412</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>18</xdr:col>
+      <xdr:col>17</xdr:col>
       <xdr:colOff>672087</xdr:colOff>
       <xdr:row>113</xdr:row>
       <xdr:rowOff>98079</xdr:rowOff>
@@ -794,13 +788,13 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>11</xdr:col>
+      <xdr:col>10</xdr:col>
       <xdr:colOff>33616</xdr:colOff>
       <xdr:row>7</xdr:row>
       <xdr:rowOff>1</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>15</xdr:col>
+      <xdr:col>14</xdr:col>
       <xdr:colOff>741314</xdr:colOff>
       <xdr:row>29</xdr:row>
       <xdr:rowOff>16844</xdr:rowOff>
@@ -1102,23 +1096,23 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:U116"/>
+  <dimension ref="A1:T116"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="5" style="1" customWidth="1"/>
     <col min="2" max="2" width="40.7109375" style="3" customWidth="1"/>
     <col min="3" max="3" width="27.5703125" style="3" bestFit="1" customWidth="1"/>
-    <col min="4" max="5" width="23.42578125" style="3" bestFit="1" customWidth="1"/>
-    <col min="6" max="121" width="12.7109375" style="3" customWidth="1"/>
-    <col min="122" max="16384" width="9.140625" style="3"/>
+    <col min="4" max="4" width="23.42578125" style="3" bestFit="1" customWidth="1"/>
+    <col min="5" max="120" width="12.7109375" style="3" customWidth="1"/>
+    <col min="121" max="16384" width="9.140625" style="3"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:12">
+    <row r="1" spans="2:11">
       <c r="B1" s="2" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="2:12">
+    <row r="2" spans="2:11">
       <c r="B2" s="4" t="s">
         <v>1</v>
       </c>
@@ -1126,14 +1120,13 @@
         <v>49</v>
       </c>
       <c r="D2" s="6"/>
-      <c r="E2" s="6"/>
+      <c r="E2" s="7"/>
       <c r="F2" s="7"/>
       <c r="G2" s="7"/>
       <c r="H2" s="7"/>
       <c r="I2" s="7"/>
-      <c r="J2" s="7"/>
-    </row>
-    <row r="3" spans="2:12">
+    </row>
+    <row r="3" spans="2:11">
       <c r="B3" s="4" t="s">
         <v>2</v>
       </c>
@@ -1141,14 +1134,13 @@
         <v>50</v>
       </c>
       <c r="D3" s="6"/>
-      <c r="E3" s="6"/>
+      <c r="E3" s="7"/>
       <c r="F3" s="7"/>
       <c r="G3" s="7"/>
       <c r="H3" s="7"/>
       <c r="I3" s="7"/>
-      <c r="J3" s="7"/>
-    </row>
-    <row r="4" spans="2:12" ht="15.75" thickBot="1">
+    </row>
+    <row r="4" spans="2:11" ht="15.75" thickBot="1">
       <c r="B4" s="8" t="s">
         <v>3</v>
       </c>
@@ -1156,46 +1148,44 @@
         <v>51</v>
       </c>
       <c r="D4" s="10"/>
-      <c r="E4" s="10"/>
+      <c r="E4" s="11"/>
       <c r="F4" s="11"/>
       <c r="G4" s="11"/>
       <c r="H4" s="11"/>
       <c r="I4" s="11"/>
-      <c r="J4" s="11"/>
-    </row>
-    <row r="5" spans="2:12">
+    </row>
+    <row r="5" spans="2:11">
       <c r="B5" s="12" t="s">
         <v>4</v>
       </c>
       <c r="C5" s="13"/>
       <c r="D5" s="13"/>
-      <c r="E5" s="13"/>
+      <c r="E5" s="14"/>
       <c r="F5" s="14"/>
       <c r="G5" s="14"/>
       <c r="H5" s="14"/>
       <c r="I5" s="14"/>
-      <c r="J5" s="14"/>
-    </row>
-    <row r="6" spans="2:12">
+    </row>
+    <row r="6" spans="2:11">
       <c r="B6" s="15"/>
     </row>
-    <row r="7" spans="2:12">
+    <row r="7" spans="2:11">
       <c r="B7" s="16" t="s">
         <v>5</v>
       </c>
-      <c r="L7" s="16" t="s">
+      <c r="K7" s="16" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="8" spans="2:12">
+    <row r="8" spans="2:11">
       <c r="B8" s="17" t="s">
         <v>7</v>
       </c>
-      <c r="C8" s="55" t="s">
+      <c r="C8" s="54" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="9" spans="2:12">
+    <row r="9" spans="2:11">
       <c r="B9" s="3" t="s">
         <v>9</v>
       </c>
@@ -1203,7 +1193,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="10" spans="2:12">
+    <row r="10" spans="2:11">
       <c r="B10" s="3" t="s">
         <v>10</v>
       </c>
@@ -1211,46 +1201,39 @@
         <v>53</v>
       </c>
     </row>
-    <row r="11" spans="2:12">
+    <row r="11" spans="2:11">
       <c r="B11" s="3" t="s">
         <v>11</v>
       </c>
       <c r="C11" s="19" t="s">
         <v>54</v>
       </c>
-      <c r="F11" s="20"/>
-    </row>
-    <row r="12" spans="2:12">
-      <c r="E12" s="21"/>
-    </row>
-    <row r="13" spans="2:12">
+      <c r="E11" s="20"/>
+    </row>
+    <row r="13" spans="2:11">
       <c r="B13" s="16" t="s">
         <v>12</v>
       </c>
-      <c r="E13" s="21"/>
-    </row>
-    <row r="14" spans="2:12">
+    </row>
+    <row r="14" spans="2:11">
       <c r="B14" s="17" t="s">
         <v>7</v>
       </c>
-      <c r="C14" s="55" t="s">
+      <c r="C14" s="54" t="s">
         <v>13</v>
       </c>
-      <c r="D14" s="55" t="s">
+      <c r="D14" s="54" t="s">
         <v>14</v>
       </c>
-      <c r="E14" s="55" t="s">
-        <v>66</v>
-      </c>
-      <c r="F14" s="17" t="s">
+      <c r="E14" s="17" t="s">
         <v>16</v>
       </c>
+      <c r="F14" s="17"/>
       <c r="G14" s="17"/>
       <c r="H14" s="17"/>
       <c r="I14" s="17"/>
-      <c r="J14" s="17"/>
-    </row>
-    <row r="15" spans="2:12">
+    </row>
+    <row r="15" spans="2:11">
       <c r="B15" s="22" t="s">
         <v>17</v>
       </c>
@@ -1260,16 +1243,13 @@
       <c r="D15" s="19" t="s">
         <v>65</v>
       </c>
-      <c r="E15" s="19" t="s">
-        <v>66</v>
-      </c>
+      <c r="E15" s="23"/>
       <c r="F15" s="23"/>
-      <c r="G15" s="23"/>
+      <c r="G15" s="24"/>
       <c r="H15" s="24"/>
       <c r="I15" s="24"/>
-      <c r="J15" s="24"/>
-    </row>
-    <row r="16" spans="2:12">
+    </row>
+    <row r="16" spans="2:11">
       <c r="B16" s="3" t="s">
         <v>18</v>
       </c>
@@ -1279,12 +1259,9 @@
       <c r="D16" s="25" t="s">
         <v>63</v>
       </c>
-      <c r="E16" s="25" t="s">
-        <v>66</v>
-      </c>
-      <c r="F16" s="21"/>
-    </row>
-    <row r="17" spans="1:21">
+      <c r="E16" s="21"/>
+    </row>
+    <row r="17" spans="1:20">
       <c r="B17" s="26" t="s">
         <v>19</v>
       </c>
@@ -1295,15 +1272,12 @@
         <f>C17</f>
         <v>{{Spot Price}}</v>
       </c>
-      <c r="E17" s="20" t="s">
-        <v>66</v>
-      </c>
-      <c r="F17" s="27"/>
+      <c r="E17" s="27"/>
+      <c r="G17" s="28"/>
       <c r="H17" s="28"/>
       <c r="I17" s="28"/>
-      <c r="J17" s="28"/>
-    </row>
-    <row r="18" spans="1:21">
+    </row>
+    <row r="18" spans="1:20">
       <c r="A18" s="1" t="s">
         <v>20</v>
       </c>
@@ -1317,21 +1291,18 @@
         <f>C18</f>
         <v>{{Spot Price}}</v>
       </c>
-      <c r="E18" s="20" t="s">
-        <v>66</v>
-      </c>
-      <c r="F18" s="27"/>
+      <c r="E18" s="27"/>
+      <c r="G18" s="28"/>
       <c r="H18" s="28"/>
       <c r="I18" s="28"/>
-      <c r="J18" s="28"/>
+      <c r="Q18" s="1" t="s">
+        <v>22</v>
+      </c>
       <c r="R18" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="S18" s="1" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="19" spans="1:21">
+    <row r="19" spans="1:20">
       <c r="A19" s="1" t="s">
         <v>24</v>
       </c>
@@ -1345,21 +1316,18 @@
         <f>C19</f>
         <v>{{Time to Maturity}}</v>
       </c>
-      <c r="E19" s="20" t="s">
-        <v>66</v>
-      </c>
-      <c r="F19" s="27"/>
+      <c r="E19" s="27"/>
+      <c r="G19" s="28"/>
       <c r="H19" s="28"/>
       <c r="I19" s="28"/>
-      <c r="J19" s="28"/>
-      <c r="R19" s="3">
+      <c r="Q19" s="3">
         <v>7</v>
       </c>
-      <c r="S19" s="29">
+      <c r="R19" s="29">
         <v>3.3750000000000002E-2</v>
       </c>
     </row>
-    <row r="20" spans="1:21">
+    <row r="20" spans="1:20">
       <c r="A20" s="1" t="s">
         <v>26</v>
       </c>
@@ -1373,20 +1341,17 @@
         <f>$C$20</f>
         <v>{{Volatility}}</v>
       </c>
-      <c r="E20" s="30" t="s">
-        <v>66</v>
-      </c>
-      <c r="F20" s="21" t="s">
+      <c r="E20" s="21" t="s">
         <v>28</v>
       </c>
-      <c r="R20" s="31">
+      <c r="Q20" s="31">
         <v>10</v>
       </c>
-      <c r="S20" s="32">
+      <c r="R20" s="32">
         <v>3.4099999999999998E-2</v>
       </c>
     </row>
-    <row r="21" spans="1:21">
+    <row r="21" spans="1:20">
       <c r="A21" s="1" t="s">
         <v>29</v>
       </c>
@@ -1400,20 +1365,17 @@
         <f>C21</f>
         <v>{{Risk-free Rate}}</v>
       </c>
-      <c r="E21" s="33" t="s">
-        <v>66</v>
-      </c>
-      <c r="F21" s="21"/>
-      <c r="R21" s="20" t="str">
+      <c r="E21" s="21"/>
+      <c r="Q21" s="20" t="str">
         <f>C19</f>
         <v>{{Time to Maturity}}</v>
       </c>
-      <c r="S21" s="30" t="e">
-        <f>TREND(S19:S20,R19:R20,R21)</f>
+      <c r="R21" s="30" t="e">
+        <f>TREND(R19:R20,Q19:Q20,Q21)</f>
         <v>#VALUE!</v>
       </c>
     </row>
-    <row r="22" spans="1:21">
+    <row r="22" spans="1:20">
       <c r="A22" s="1" t="s">
         <v>31</v>
       </c>
@@ -1427,12 +1389,9 @@
         <f>$C$22</f>
         <v>{{Dividend Yield}}</v>
       </c>
-      <c r="E22" s="30" t="s">
-        <v>66</v>
-      </c>
-      <c r="F22" s="21"/>
-    </row>
-    <row r="23" spans="1:21">
+      <c r="E22" s="21"/>
+    </row>
+    <row r="23" spans="1:20">
       <c r="A23" s="1" t="s">
         <v>33</v>
       </c>
@@ -1446,14 +1405,11 @@
         <f>$C$23</f>
         <v>{{Exercise Multiple}}</v>
       </c>
-      <c r="E23" s="34" t="s">
-        <v>66</v>
-      </c>
-      <c r="F23" s="21" t="s">
+      <c r="E23" s="21" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="24" spans="1:21">
+    <row r="24" spans="1:20">
       <c r="B24" s="26" t="s">
         <v>36</v>
       </c>
@@ -1464,12 +1420,9 @@
         <f>$C$24</f>
         <v>0</v>
       </c>
-      <c r="E24" s="30" t="s">
-        <v>66</v>
-      </c>
-      <c r="F24" s="21"/>
-    </row>
-    <row r="25" spans="1:21">
+      <c r="E24" s="21"/>
+    </row>
+    <row r="25" spans="1:20">
       <c r="B25" s="26" t="s">
         <v>37</v>
       </c>
@@ -1480,49 +1433,40 @@
         <f>C25</f>
         <v>{{Post-vesting Exit Rate}}</v>
       </c>
-      <c r="E25" s="35" t="s">
-        <v>66</v>
-      </c>
-      <c r="F25" s="21" t="s">
+      <c r="E25" s="21" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="26" spans="1:21">
+    <row r="26" spans="1:20">
       <c r="B26" s="36" t="s">
         <v>39</v>
       </c>
       <c r="C26" s="37" t="s">
+        <v>68</v>
+      </c>
+      <c r="D26" s="37" t="s">
         <v>69</v>
       </c>
-      <c r="D26" s="37" t="s">
-        <v>70</v>
-      </c>
-      <c r="E26" s="37" t="s">
-        <v>66</v>
-      </c>
-      <c r="F26" s="31"/>
-      <c r="G26" s="38"/>
-    </row>
-    <row r="27" spans="1:21">
+      <c r="E26" s="31"/>
+      <c r="F26" s="38"/>
+    </row>
+    <row r="27" spans="1:20">
       <c r="B27" s="39" t="s">
         <v>40</v>
       </c>
       <c r="C27" s="40" t="s">
+        <v>66</v>
+      </c>
+      <c r="D27" s="40" t="s">
         <v>67</v>
       </c>
-      <c r="D27" s="40" t="s">
-        <v>68</v>
-      </c>
-      <c r="E27" s="40" t="s">
-        <v>66</v>
-      </c>
-      <c r="F27" s="41"/>
+      <c r="E27" s="41"/>
+      <c r="F27" s="42"/>
       <c r="G27" s="42"/>
       <c r="H27" s="42"/>
       <c r="I27" s="42"/>
-      <c r="J27" s="42"/>
-    </row>
-    <row r="28" spans="1:21" ht="15.75" thickBot="1">
+    </row>
+    <row r="28" spans="1:20" ht="15.75" thickBot="1">
       <c r="B28" s="43" t="s">
         <v>41</v>
       </c>
@@ -1534,16 +1478,13 @@
         <f>D27*D15</f>
         <v>#VALUE!</v>
       </c>
-      <c r="E28" s="44" t="s">
-        <v>66</v>
-      </c>
-      <c r="F28" s="45"/>
+      <c r="E28" s="45"/>
+      <c r="F28" s="46"/>
       <c r="G28" s="46"/>
       <c r="H28" s="46"/>
       <c r="I28" s="46"/>
-      <c r="J28" s="46"/>
-    </row>
-    <row r="29" spans="1:21" ht="15.75" thickTop="1">
+    </row>
+    <row r="29" spans="1:20" ht="15.75" thickTop="1">
       <c r="B29" s="47"/>
       <c r="C29" s="48" t="e">
         <f>C27/C17</f>
@@ -1553,40 +1494,36 @@
         <f>D27/D17</f>
         <v>#VALUE!</v>
       </c>
-      <c r="E29" s="48" t="s">
-        <v>66</v>
-      </c>
+      <c r="E29" s="47"/>
       <c r="F29" s="47"/>
       <c r="G29" s="47"/>
       <c r="H29" s="47"/>
       <c r="I29" s="47"/>
-      <c r="J29" s="47"/>
-    </row>
-    <row r="30" spans="1:21">
+    </row>
+    <row r="30" spans="1:20">
       <c r="B30" s="47"/>
       <c r="C30" s="48"/>
       <c r="D30" s="48"/>
-      <c r="E30" s="48"/>
+      <c r="E30" s="47"/>
       <c r="F30" s="47"/>
       <c r="G30" s="47"/>
       <c r="H30" s="47"/>
       <c r="I30" s="47"/>
-      <c r="J30" s="47"/>
-    </row>
-    <row r="31" spans="1:21" s="47" customFormat="1">
+    </row>
+    <row r="31" spans="1:20" s="47" customFormat="1">
       <c r="A31" s="49"/>
       <c r="B31" s="50"/>
       <c r="C31" s="51"/>
       <c r="D31" s="50"/>
-      <c r="E31" s="52"/>
+      <c r="E31" s="50"/>
       <c r="F31" s="50"/>
       <c r="G31" s="50"/>
       <c r="H31" s="50"/>
       <c r="I31" s="50"/>
-      <c r="J31" s="50"/>
-      <c r="L31" s="16" t="s">
+      <c r="K31" s="16" t="s">
         <v>42</v>
       </c>
+      <c r="L31" s="3"/>
       <c r="M31" s="3"/>
       <c r="N31" s="3"/>
       <c r="O31" s="3"/>
@@ -1595,16 +1532,16 @@
       <c r="R31" s="3"/>
       <c r="S31" s="3"/>
       <c r="T31" s="3"/>
-      <c r="U31" s="3"/>
-    </row>
-    <row r="32" spans="1:21" s="50" customFormat="1">
-      <c r="A32" s="53"/>
-      <c r="B32" s="54"/>
+    </row>
+    <row r="32" spans="1:20" s="50" customFormat="1">
+      <c r="A32" s="52"/>
+      <c r="B32" s="53"/>
+      <c r="E32" s="3"/>
       <c r="F32" s="3"/>
       <c r="G32" s="3"/>
       <c r="H32" s="3"/>
       <c r="I32" s="3"/>
-      <c r="J32" s="3"/>
+      <c r="K32" s="3"/>
       <c r="L32" s="3"/>
       <c r="M32" s="3"/>
       <c r="N32" s="3"/>
@@ -1613,233 +1550,185 @@
       <c r="Q32" s="3"/>
       <c r="R32" s="3"/>
       <c r="S32" s="3"/>
-      <c r="T32" s="3"/>
-      <c r="U32" s="47"/>
-    </row>
-    <row r="33" spans="2:21">
-      <c r="B33" s="54"/>
-      <c r="C33" s="54"/>
-      <c r="U33" s="50"/>
-    </row>
-    <row r="34" spans="2:21">
-      <c r="B34" s="54"/>
-      <c r="C34" s="54"/>
-    </row>
-    <row r="35" spans="2:21">
-      <c r="B35" s="54"/>
-      <c r="C35" s="54"/>
-      <c r="D35" s="54"/>
-      <c r="E35" s="54"/>
-    </row>
-    <row r="36" spans="2:21">
-      <c r="B36" s="54"/>
-      <c r="C36" s="54"/>
-      <c r="D36" s="54"/>
-      <c r="E36" s="54"/>
-    </row>
-    <row r="37" spans="2:21">
-      <c r="B37" s="54"/>
-      <c r="C37" s="54"/>
-      <c r="D37" s="54"/>
-      <c r="E37" s="54"/>
-    </row>
-    <row r="39" spans="2:21" hidden="1">
+      <c r="T32" s="47"/>
+    </row>
+    <row r="33" spans="2:20">
+      <c r="B33" s="53"/>
+      <c r="C33" s="53"/>
+      <c r="T33" s="50"/>
+    </row>
+    <row r="34" spans="2:20">
+      <c r="B34" s="53"/>
+      <c r="C34" s="53"/>
+    </row>
+    <row r="35" spans="2:20">
+      <c r="B35" s="53"/>
+      <c r="C35" s="53"/>
+      <c r="D35" s="53"/>
+    </row>
+    <row r="36" spans="2:20">
+      <c r="B36" s="53"/>
+      <c r="C36" s="53"/>
+      <c r="D36" s="53"/>
+    </row>
+    <row r="37" spans="2:20">
+      <c r="B37" s="53"/>
+      <c r="C37" s="53"/>
+      <c r="D37" s="53"/>
+    </row>
+    <row r="39" spans="2:20" hidden="1">
       <c r="C39" s="3" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="40" spans="2:21" hidden="1">
-      <c r="C40" s="54" t="e">
+    <row r="40" spans="2:20" hidden="1">
+      <c r="C40" s="53" t="e">
         <f>#REF!</f>
         <v>#REF!</v>
       </c>
     </row>
-    <row r="41" spans="2:21" hidden="1">
-      <c r="B41" s="54">
+    <row r="41" spans="2:20" hidden="1">
+      <c r="B41" s="53">
         <v>8.8000000000000007</v>
       </c>
-      <c r="C41" s="54" t="e">
-        <v>#REF!</v>
-      </c>
-      <c r="D41" s="54"/>
-      <c r="E41" s="54">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="42" spans="2:21" hidden="1">
-      <c r="B42" s="54">
+      <c r="C41" s="53" t="e">
+        <v>#REF!</v>
+      </c>
+      <c r="D41" s="53"/>
+    </row>
+    <row r="42" spans="2:20" hidden="1">
+      <c r="B42" s="53">
         <f>B41+1</f>
         <v>9.8000000000000007</v>
       </c>
-      <c r="C42" s="54" t="e">
-        <v>#REF!</v>
-      </c>
-      <c r="D42" s="54"/>
-      <c r="E42" s="54">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="43" spans="2:21" hidden="1">
-      <c r="B43" s="54">
+      <c r="C42" s="53" t="e">
+        <v>#REF!</v>
+      </c>
+      <c r="D42" s="53"/>
+    </row>
+    <row r="43" spans="2:20" hidden="1">
+      <c r="B43" s="53">
         <f t="shared" ref="B43:B46" si="0">B42+1</f>
         <v>10.8</v>
       </c>
-      <c r="C43" s="54" t="e">
-        <v>#REF!</v>
-      </c>
-      <c r="D43" s="54"/>
-      <c r="E43" s="54">
-        <v>5</v>
-      </c>
-      <c r="L43" s="16" t="s">
+      <c r="C43" s="53" t="e">
+        <v>#REF!</v>
+      </c>
+      <c r="D43" s="53"/>
+      <c r="K43" s="16" t="s">
         <v>43</v>
       </c>
     </row>
-    <row r="44" spans="2:21" hidden="1">
-      <c r="B44" s="54">
+    <row r="44" spans="2:20" hidden="1">
+      <c r="B44" s="53">
         <f t="shared" si="0"/>
         <v>11.8</v>
       </c>
-      <c r="C44" s="54" t="e">
-        <v>#REF!</v>
-      </c>
-      <c r="D44" s="54"/>
-      <c r="E44" s="54">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="45" spans="2:21" hidden="1">
-      <c r="B45" s="54">
+      <c r="C44" s="53" t="e">
+        <v>#REF!</v>
+      </c>
+      <c r="D44" s="53"/>
+    </row>
+    <row r="45" spans="2:20" hidden="1">
+      <c r="B45" s="53">
         <f t="shared" si="0"/>
         <v>12.8</v>
       </c>
-      <c r="C45" s="54" t="e">
-        <v>#REF!</v>
-      </c>
-      <c r="D45" s="54"/>
-      <c r="E45" s="54">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="46" spans="2:21" hidden="1">
-      <c r="B46" s="54">
+      <c r="C45" s="53" t="e">
+        <v>#REF!</v>
+      </c>
+      <c r="D45" s="53"/>
+    </row>
+    <row r="46" spans="2:20" hidden="1">
+      <c r="B46" s="53">
         <f t="shared" si="0"/>
         <v>13.8</v>
       </c>
-      <c r="C46" s="54" t="e">
-        <v>#REF!</v>
-      </c>
-      <c r="D46" s="54"/>
-      <c r="E46" s="54">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="47" spans="2:21" hidden="1">
-      <c r="E47" s="54">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="48" spans="2:21" hidden="1">
+      <c r="C46" s="53" t="e">
+        <v>#REF!</v>
+      </c>
+      <c r="D46" s="53"/>
+    </row>
+    <row r="47" spans="2:20" hidden="1"/>
+    <row r="48" spans="2:20" hidden="1">
       <c r="C48" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="E48" s="54">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="49" spans="2:20" hidden="1">
-      <c r="C49" s="54" t="e">
+    </row>
+    <row r="49" spans="2:19" hidden="1">
+      <c r="C49" s="53" t="e">
         <f>#REF!</f>
         <v>#REF!</v>
       </c>
-      <c r="E49" s="54"/>
-    </row>
-    <row r="50" spans="2:20" hidden="1">
-      <c r="B50" s="54">
+    </row>
+    <row r="50" spans="2:19" hidden="1">
+      <c r="B50" s="53">
         <v>8.8000000000000007</v>
       </c>
-      <c r="C50" s="54" t="e">
-        <v>#REF!</v>
-      </c>
-      <c r="D50" s="54"/>
-    </row>
-    <row r="51" spans="2:20" hidden="1">
-      <c r="B51" s="54">
+      <c r="C50" s="53" t="e">
+        <v>#REF!</v>
+      </c>
+      <c r="D50" s="53"/>
+    </row>
+    <row r="51" spans="2:19" hidden="1">
+      <c r="B51" s="53">
         <f>B50+1</f>
         <v>9.8000000000000007</v>
       </c>
-      <c r="C51" s="54" t="e">
-        <v>#REF!</v>
-      </c>
-      <c r="D51" s="54"/>
-      <c r="L51" s="16" t="s">
+      <c r="C51" s="53" t="e">
+        <v>#REF!</v>
+      </c>
+      <c r="D51" s="53"/>
+      <c r="K51" s="16" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="52" spans="2:20" hidden="1">
-      <c r="B52" s="54">
+    <row r="52" spans="2:19" hidden="1">
+      <c r="B52" s="53">
         <f t="shared" ref="B52:B55" si="1">B51+1</f>
         <v>10.8</v>
       </c>
-      <c r="C52" s="54" t="e">
-        <v>#REF!</v>
-      </c>
-      <c r="D52" s="54"/>
-      <c r="E52" s="54">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="53" spans="2:20" hidden="1">
-      <c r="B53" s="54">
+      <c r="C52" s="53" t="e">
+        <v>#REF!</v>
+      </c>
+      <c r="D52" s="53"/>
+    </row>
+    <row r="53" spans="2:19" hidden="1">
+      <c r="B53" s="53">
         <f t="shared" si="1"/>
         <v>11.8</v>
       </c>
-      <c r="C53" s="54" t="e">
-        <v>#REF!</v>
-      </c>
-      <c r="D53" s="54"/>
-      <c r="E53" s="54">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="54" spans="2:20" hidden="1">
-      <c r="B54" s="54">
+      <c r="C53" s="53" t="e">
+        <v>#REF!</v>
+      </c>
+      <c r="D53" s="53"/>
+    </row>
+    <row r="54" spans="2:19" hidden="1">
+      <c r="B54" s="53">
         <f t="shared" si="1"/>
         <v>12.8</v>
       </c>
-      <c r="C54" s="54" t="e">
-        <v>#REF!</v>
-      </c>
-      <c r="D54" s="54"/>
-      <c r="E54" s="54">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="55" spans="2:20" hidden="1">
-      <c r="B55" s="54">
+      <c r="C54" s="53" t="e">
+        <v>#REF!</v>
+      </c>
+      <c r="D54" s="53"/>
+    </row>
+    <row r="55" spans="2:19" hidden="1">
+      <c r="B55" s="53">
         <f t="shared" si="1"/>
         <v>13.8</v>
       </c>
-      <c r="C55" s="54" t="e">
-        <v>#REF!</v>
-      </c>
-      <c r="D55" s="54"/>
-      <c r="E55" s="54">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="56" spans="2:20" hidden="1">
-      <c r="E56" s="54">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="57" spans="2:20" hidden="1">
+      <c r="C55" s="53" t="e">
+        <v>#REF!</v>
+      </c>
+      <c r="D55" s="53"/>
+    </row>
+    <row r="56" spans="2:19" hidden="1"/>
+    <row r="57" spans="2:19" hidden="1">
       <c r="C57" s="3" t="s">
         <v>45</v>
       </c>
-      <c r="E57" s="54">
-        <v>9</v>
-      </c>
+      <c r="K57" s="47"/>
       <c r="L57" s="47"/>
       <c r="M57" s="47"/>
       <c r="N57" s="47"/>
@@ -1848,16 +1737,13 @@
       <c r="Q57" s="47"/>
       <c r="R57" s="47"/>
       <c r="S57" s="47"/>
-      <c r="T57" s="47"/>
-    </row>
-    <row r="58" spans="2:20" hidden="1">
-      <c r="C58" s="54" t="e">
+    </row>
+    <row r="58" spans="2:19" hidden="1">
+      <c r="C58" s="53" t="e">
         <f>#REF!</f>
         <v>#REF!</v>
       </c>
-      <c r="E58" s="54">
-        <v>10</v>
-      </c>
+      <c r="K58" s="50"/>
       <c r="L58" s="50"/>
       <c r="M58" s="50"/>
       <c r="N58" s="50"/>
@@ -1866,174 +1752,141 @@
       <c r="Q58" s="50"/>
       <c r="R58" s="50"/>
       <c r="S58" s="50"/>
-      <c r="T58" s="50"/>
-    </row>
-    <row r="59" spans="2:20" hidden="1">
-      <c r="B59" s="54">
+    </row>
+    <row r="59" spans="2:19" hidden="1">
+      <c r="B59" s="53">
         <v>8.8000000000000007</v>
       </c>
-      <c r="C59" s="54" t="e">
-        <v>#REF!</v>
-      </c>
-      <c r="D59" s="54"/>
-    </row>
-    <row r="60" spans="2:20" hidden="1">
-      <c r="B60" s="54">
+      <c r="C59" s="53" t="e">
+        <v>#REF!</v>
+      </c>
+      <c r="D59" s="53"/>
+    </row>
+    <row r="60" spans="2:19" hidden="1">
+      <c r="B60" s="53">
         <f>B59+1</f>
         <v>9.8000000000000007</v>
       </c>
-      <c r="C60" s="54" t="e">
-        <v>#REF!</v>
-      </c>
-      <c r="D60" s="54"/>
-    </row>
-    <row r="61" spans="2:20" hidden="1">
-      <c r="B61" s="54">
+      <c r="C60" s="53" t="e">
+        <v>#REF!</v>
+      </c>
+      <c r="D60" s="53"/>
+    </row>
+    <row r="61" spans="2:19" hidden="1">
+      <c r="B61" s="53">
         <f t="shared" ref="B61:B64" si="2">B60+1</f>
         <v>10.8</v>
       </c>
-      <c r="C61" s="54" t="e">
-        <v>#REF!</v>
-      </c>
-      <c r="D61" s="54"/>
-      <c r="L61" s="16" t="s">
+      <c r="C61" s="53" t="e">
+        <v>#REF!</v>
+      </c>
+      <c r="D61" s="53"/>
+      <c r="K61" s="16" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="62" spans="2:20" hidden="1">
-      <c r="B62" s="54">
+    <row r="62" spans="2:19" hidden="1">
+      <c r="B62" s="53">
         <f t="shared" si="2"/>
         <v>11.8</v>
       </c>
-      <c r="C62" s="54" t="e">
-        <v>#REF!</v>
-      </c>
-      <c r="D62" s="54"/>
-      <c r="E62" s="54">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="63" spans="2:20" hidden="1">
-      <c r="B63" s="54">
+      <c r="C62" s="53" t="e">
+        <v>#REF!</v>
+      </c>
+      <c r="D62" s="53"/>
+    </row>
+    <row r="63" spans="2:19" hidden="1">
+      <c r="B63" s="53">
         <f t="shared" si="2"/>
         <v>12.8</v>
       </c>
-      <c r="C63" s="54" t="e">
-        <v>#REF!</v>
-      </c>
-      <c r="D63" s="54"/>
-      <c r="E63" s="54">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="64" spans="2:20" hidden="1">
-      <c r="B64" s="54">
+      <c r="C63" s="53" t="e">
+        <v>#REF!</v>
+      </c>
+      <c r="D63" s="53"/>
+    </row>
+    <row r="64" spans="2:19" hidden="1">
+      <c r="B64" s="53">
         <f t="shared" si="2"/>
         <v>13.8</v>
       </c>
-      <c r="C64" s="54" t="e">
-        <v>#REF!</v>
-      </c>
-      <c r="D64" s="54"/>
-      <c r="E64" s="54">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="65" spans="2:12" hidden="1">
-      <c r="E65" s="54">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="66" spans="2:12" hidden="1">
-      <c r="E66" s="54">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="67" spans="2:12" hidden="1">
-      <c r="E67" s="54">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="68" spans="2:12" hidden="1"/>
-    <row r="69" spans="2:12">
+      <c r="C64" s="53" t="e">
+        <v>#REF!</v>
+      </c>
+      <c r="D64" s="53"/>
+    </row>
+    <row r="65" spans="2:11" hidden="1"/>
+    <row r="66" spans="2:11" hidden="1"/>
+    <row r="67" spans="2:11" hidden="1"/>
+    <row r="68" spans="2:11" hidden="1"/>
+    <row r="69" spans="2:11">
       <c r="B69" s="47"/>
       <c r="C69" s="47"/>
       <c r="D69" s="47"/>
-      <c r="E69" s="47"/>
-      <c r="L69" s="16" t="s">
+      <c r="K69" s="16" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="70" spans="2:12">
+    <row r="70" spans="2:11">
       <c r="B70" s="50"/>
       <c r="C70" s="51"/>
       <c r="D70" s="51"/>
-      <c r="E70" s="51"/>
-    </row>
-    <row r="71" spans="2:12">
-      <c r="B71" s="54"/>
-      <c r="C71" s="54"/>
-      <c r="D71" s="54"/>
-      <c r="E71" s="54"/>
-    </row>
-    <row r="72" spans="2:12">
-      <c r="B72" s="54"/>
-      <c r="C72" s="54"/>
-      <c r="D72" s="54"/>
-      <c r="E72" s="54"/>
-    </row>
-    <row r="73" spans="2:12">
-      <c r="B73" s="54"/>
-      <c r="C73" s="54"/>
-      <c r="D73" s="54"/>
-      <c r="E73" s="54"/>
-    </row>
-    <row r="74" spans="2:12">
-      <c r="B74" s="54"/>
-      <c r="C74" s="54"/>
-      <c r="D74" s="54"/>
-      <c r="E74" s="54"/>
-    </row>
-    <row r="75" spans="2:12">
-      <c r="B75" s="54"/>
-      <c r="C75" s="54"/>
-      <c r="D75" s="54"/>
-      <c r="E75" s="54"/>
-    </row>
-    <row r="76" spans="2:12">
-      <c r="B76" s="54"/>
-      <c r="C76" s="54"/>
-      <c r="D76" s="54"/>
-      <c r="E76" s="54"/>
-    </row>
-    <row r="77" spans="2:12">
-      <c r="B77" s="54"/>
-      <c r="C77" s="54"/>
-      <c r="D77" s="54"/>
-      <c r="E77" s="54"/>
-    </row>
-    <row r="78" spans="2:12">
-      <c r="B78" s="54"/>
-      <c r="C78" s="54"/>
-      <c r="D78" s="54"/>
-      <c r="E78" s="54"/>
-    </row>
-    <row r="79" spans="2:12">
-      <c r="B79" s="54"/>
-      <c r="C79" s="54"/>
-      <c r="D79" s="54"/>
-      <c r="E79" s="54"/>
-      <c r="L79" s="16" t="s">
+    </row>
+    <row r="71" spans="2:11">
+      <c r="B71" s="53"/>
+      <c r="C71" s="53"/>
+      <c r="D71" s="53"/>
+    </row>
+    <row r="72" spans="2:11">
+      <c r="B72" s="53"/>
+      <c r="C72" s="53"/>
+      <c r="D72" s="53"/>
+    </row>
+    <row r="73" spans="2:11">
+      <c r="B73" s="53"/>
+      <c r="C73" s="53"/>
+      <c r="D73" s="53"/>
+    </row>
+    <row r="74" spans="2:11">
+      <c r="B74" s="53"/>
+      <c r="C74" s="53"/>
+      <c r="D74" s="53"/>
+    </row>
+    <row r="75" spans="2:11">
+      <c r="B75" s="53"/>
+      <c r="C75" s="53"/>
+      <c r="D75" s="53"/>
+    </row>
+    <row r="76" spans="2:11">
+      <c r="B76" s="53"/>
+      <c r="C76" s="53"/>
+      <c r="D76" s="53"/>
+    </row>
+    <row r="77" spans="2:11">
+      <c r="B77" s="53"/>
+      <c r="C77" s="53"/>
+      <c r="D77" s="53"/>
+    </row>
+    <row r="78" spans="2:11">
+      <c r="B78" s="53"/>
+      <c r="C78" s="53"/>
+      <c r="D78" s="53"/>
+    </row>
+    <row r="79" spans="2:11">
+      <c r="B79" s="53"/>
+      <c r="C79" s="53"/>
+      <c r="D79" s="53"/>
+      <c r="K79" s="16" t="s">
         <v>43</v>
       </c>
     </row>
-    <row r="91" spans="12:12">
-      <c r="L91" s="16" t="s">
+    <row r="91" spans="11:11">
+      <c r="K91" s="16" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="116" spans="12:12">
-      <c r="L116" s="16" t="s">
+    <row r="116" spans="11:11">
+      <c r="K116" s="16" t="s">
         <v>48</v>
       </c>
     </row>

</xml_diff>